<commit_message>
Lead The Corner Hengelo toegevoegd aan leadlijst
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CXZAe6mJ9JKuTqwEhBfQPp
</commit_message>
<xml_diff>
--- a/klantenwerving/leads-hengelo-zonder-website.xlsx
+++ b/klantenwerving/leads-hengelo-zonder-website.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4758,8 +4758,69 @@
       </c>
       <c r="M71" s="3" t="inlineStr"/>
     </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Hengelo</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>The Corner Hengelo</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>snackbar (döner, kapsalon, burgers)</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Dennenbosweg 92, 7556 Hengelo</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>nieuw, opent november 2026 (nog geen reviews)</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>flyer; tel 074 737 0119</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>1) Nieuwe zaak: site + Google-profiel vanaf dag 1, opening-actie online. 2) Menukaart + bel/route-knop op de telefoon.</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>Ik zag jullie flyer voor de opening en heb alvast een site voor The Corner gemaakt.</t>
+        </is>
+      </c>
+      <c r="L72" s="4" t="inlineStr">
+        <is>
+          <t>open in Maps</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M71"/>
+  <autoFilter ref="A1:M72"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -4831,6 +4892,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>